<commit_message>
Add verified 2026-W42 Monday player records
</commit_message>
<xml_diff>
--- a/Japanese-Players-Abroad.xlsx
+++ b/Japanese-Players-Abroad.xlsx
@@ -2,15 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="1" r:id="Ra98cca95ef674fe6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-W41" sheetId="2" r:id="R499ca74beaf24358"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-W41-Fri" sheetId="3" r:id="Re8e92575f1644616"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-W41-Sat" sheetId="4" r:id="Rdb4b8f7ce3ea43b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-W41-Sun" sheetId="5" r:id="Rb9b51c14e9e4412d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-W42" sheetId="6" r:id="R94dd6fcdf3274bba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roster Checks" sheetId="7" r:id="R639a0c5a82d84e88"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="League Coverage" sheetId="8" r:id="R53f6538221854258"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Definitions" sheetId="9" r:id="Refb45613b0fd4c3f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="1" r:id="Rbd44fb8bccda4188"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-W41" sheetId="2" r:id="Rb92557d1e95e4f4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-W41-Fri" sheetId="3" r:id="R06ee61b4d6e44dea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-W41-Sat" sheetId="4" r:id="R51e95f6513504cc9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-W41-Sun" sheetId="5" r:id="Rd8212cb08fc14eb2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-W42" sheetId="6" r:id="R430dbf448c9b4762"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roster Checks" sheetId="7" r:id="R0f7cf860774f48b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="League Coverage" sheetId="8" r:id="R14c2622d5fc340d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Definitions" sheetId="9" r:id="R69cd71607c504cbf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-W42-Mon" sheetId="10" r:id="Re28efa9c23c34831"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -37,12 +38,17 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="3">
+  <x:fills count="4">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF162B40"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -62,7 +68,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="6">
+  <x:cellXfs count="8">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -76,6 +82,12 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -98,6 +110,44 @@
     <x:tableColumn id="9" name="source_as_of"/>
     <x:tableColumn id="10" name="notes"/>
     <x:tableColumn id="11" name="affiliations"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="T2026W42Mon" displayName="T2026W42Mon" ref="A1:AD3" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="30">
+    <x:tableColumn id="1" name="week"/>
+    <x:tableColumn id="2" name="day_sheet"/>
+    <x:tableColumn id="3" name="match_id"/>
+    <x:tableColumn id="4" name="player_id"/>
+    <x:tableColumn id="5" name="name_ja"/>
+    <x:tableColumn id="6" name="name_en"/>
+    <x:tableColumn id="7" name="league"/>
+    <x:tableColumn id="8" name="club"/>
+    <x:tableColumn id="9" name="club_id"/>
+    <x:tableColumn id="10" name="home"/>
+    <x:tableColumn id="11" name="home_id"/>
+    <x:tableColumn id="12" name="away"/>
+    <x:tableColumn id="13" name="away_id"/>
+    <x:tableColumn id="14" name="home_goals"/>
+    <x:tableColumn id="15" name="away_goals"/>
+    <x:tableColumn id="16" name="kickoff_local"/>
+    <x:tableColumn id="17" name="kickoff_jst"/>
+    <x:tableColumn id="18" name="status"/>
+    <x:tableColumn id="19" name="minutes"/>
+    <x:tableColumn id="20" name="goals"/>
+    <x:tableColumn id="21" name="assists"/>
+    <x:tableColumn id="22" name="own_goals"/>
+    <x:tableColumn id="23" name="yellow_cards"/>
+    <x:tableColumn id="24" name="red_cards"/>
+    <x:tableColumn id="25" name="rating"/>
+    <x:tableColumn id="26" name="rating_provider"/>
+    <x:tableColumn id="27" name="source_url"/>
+    <x:tableColumn id="28" name="verified_at"/>
+    <x:tableColumn id="29" name="verification_status"/>
+    <x:tableColumn id="30" name="notes"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -256,7 +306,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="T2026W42" displayName="T2026W42" ref="A1:AD2" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="T2026W42" displayName="T2026W42" ref="A1:AD3" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="30">
     <x:tableColumn id="1" name="week"/>
     <x:tableColumn id="2" name="day_sheet"/>
@@ -4528,7 +4578,309 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6e24e4bc98aa4dcd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R06ef23f2d8aa4d8b"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="20" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="28" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="28" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="30" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="30" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="30" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="20" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="20" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="20" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="20" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="20" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="20" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="30" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="30" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="30" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="20" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="20" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="20" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="20" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="20" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="20" hidden="0" customWidth="1"/>
+    <x:col min="25" max="25" width="20" hidden="0" customWidth="1"/>
+    <x:col min="26" max="26" width="20" hidden="0" customWidth="1"/>
+    <x:col min="27" max="27" width="74" hidden="0" customWidth="1"/>
+    <x:col min="28" max="28" width="20" hidden="0" customWidth="1"/>
+    <x:col min="29" max="29" width="30" hidden="0" customWidth="1"/>
+    <x:col min="30" max="30" width="75" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="32" customHeight="1">
+      <x:c r="A1" s="6" t="str">
+        <x:v>week</x:v>
+      </x:c>
+      <x:c r="B1" s="6" t="str">
+        <x:v>day_sheet</x:v>
+      </x:c>
+      <x:c r="C1" s="6" t="str">
+        <x:v>match_id</x:v>
+      </x:c>
+      <x:c r="D1" s="6" t="str">
+        <x:v>player_id</x:v>
+      </x:c>
+      <x:c r="E1" s="6" t="str">
+        <x:v>name_ja</x:v>
+      </x:c>
+      <x:c r="F1" s="6" t="str">
+        <x:v>name_en</x:v>
+      </x:c>
+      <x:c r="G1" s="6" t="str">
+        <x:v>league</x:v>
+      </x:c>
+      <x:c r="H1" s="6" t="str">
+        <x:v>club</x:v>
+      </x:c>
+      <x:c r="I1" s="6" t="str">
+        <x:v>club_id</x:v>
+      </x:c>
+      <x:c r="J1" s="6" t="str">
+        <x:v>home</x:v>
+      </x:c>
+      <x:c r="K1" s="6" t="str">
+        <x:v>home_id</x:v>
+      </x:c>
+      <x:c r="L1" s="6" t="str">
+        <x:v>away</x:v>
+      </x:c>
+      <x:c r="M1" s="6" t="str">
+        <x:v>away_id</x:v>
+      </x:c>
+      <x:c r="N1" s="6" t="str">
+        <x:v>home_goals</x:v>
+      </x:c>
+      <x:c r="O1" s="6" t="str">
+        <x:v>away_goals</x:v>
+      </x:c>
+      <x:c r="P1" s="6" t="str">
+        <x:v>kickoff_local</x:v>
+      </x:c>
+      <x:c r="Q1" s="6" t="str">
+        <x:v>kickoff_jst</x:v>
+      </x:c>
+      <x:c r="R1" s="6" t="str">
+        <x:v>status</x:v>
+      </x:c>
+      <x:c r="S1" s="6" t="str">
+        <x:v>minutes</x:v>
+      </x:c>
+      <x:c r="T1" s="6" t="str">
+        <x:v>goals</x:v>
+      </x:c>
+      <x:c r="U1" s="6" t="str">
+        <x:v>assists</x:v>
+      </x:c>
+      <x:c r="V1" s="6" t="str">
+        <x:v>own_goals</x:v>
+      </x:c>
+      <x:c r="W1" s="6" t="str">
+        <x:v>yellow_cards</x:v>
+      </x:c>
+      <x:c r="X1" s="6" t="str">
+        <x:v>red_cards</x:v>
+      </x:c>
+      <x:c r="Y1" s="6" t="str">
+        <x:v>rating</x:v>
+      </x:c>
+      <x:c r="Z1" s="6" t="str">
+        <x:v>rating_provider</x:v>
+      </x:c>
+      <x:c r="AA1" s="6" t="str">
+        <x:v>source_url</x:v>
+      </x:c>
+      <x:c r="AB1" s="6" t="str">
+        <x:v>verified_at</x:v>
+      </x:c>
+      <x:c r="AC1" s="6" t="str">
+        <x:v>verification_status</x:v>
+      </x:c>
+      <x:c r="AD1" s="6" t="str">
+        <x:v>notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="25" customHeight="1">
+      <x:c r="A2" s="2" t="str">
+        <x:v>2026-W42</x:v>
+      </x:c>
+      <x:c r="B2" s="2" t="str">
+        <x:v>2026-W42-Mon</x:v>
+      </x:c>
+      <x:c r="C2" s="2" t="str">
+        <x:v>5795468</x:v>
+      </x:c>
+      <x:c r="D2" s="2" t="str">
+        <x:v>jp-007</x:v>
+      </x:c>
+      <x:c r="E2" s="2" t="str">
+        <x:v>坂元達裕</x:v>
+      </x:c>
+      <x:c r="F2" s="2" t="str">
+        <x:v>Tatsuhiro Sakamoto</x:v>
+      </x:c>
+      <x:c r="G2" s="2" t="str">
+        <x:v>Premier League</x:v>
+      </x:c>
+      <x:c r="H2" s="2" t="str">
+        <x:v>Coventry City</x:v>
+      </x:c>
+      <x:c r="I2" s="2" t="n">
+        <x:v>8669</x:v>
+      </x:c>
+      <x:c r="J2" s="2" t="str">
+        <x:v>Coventry City</x:v>
+      </x:c>
+      <x:c r="K2" s="2" t="n">
+        <x:v>8669</x:v>
+      </x:c>
+      <x:c r="L2" s="2" t="str">
+        <x:v>Newcastle United</x:v>
+      </x:c>
+      <x:c r="M2" s="2" t="n">
+        <x:v>10261</x:v>
+      </x:c>
+      <x:c r="N2" s="2" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="O2" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P2" s="2" t="d">
+        <x:v>2026-10-12T19:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="Q2" s="2" t="d">
+        <x:v>2026-10-12T19:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="R2" s="2" t="str">
+        <x:v>Substitute</x:v>
+      </x:c>
+      <x:c r="S2" s="2" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="T2" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U2" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="V2" s="2"/>
+      <x:c r="W2" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X2" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Y2" s="2" t="n">
+        <x:v>6.5</x:v>
+      </x:c>
+      <x:c r="Z2" s="2" t="str">
+        <x:v>FotMob</x:v>
+      </x:c>
+      <x:c r="AA2" s="2" t="str">
+        <x:v>https://www.fotmob.com/matches/coventry-city-vs-newcastle-united/2yooc8#5795468</x:v>
+      </x:c>
+      <x:c r="AB2" s="2" t="str">
+        <x:v>2026-10-13</x:v>
+      </x:c>
+      <x:c r="AC2" s="2" t="str">
+        <x:v>Verified match record</x:v>
+      </x:c>
+      <x:c r="AD2" s="2" t="str">
+        <x:v>Cross-checked score and goal events: https://www.newcastleunited.com/en/news/coventry-city-a-26-27-report; minutes, assists, cards and rating: FotMob</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="25" customHeight="1">
+      <x:c r="A3" s="2" t="str">
+        <x:v>2026-W42</x:v>
+      </x:c>
+      <x:c r="B3" s="2" t="str">
+        <x:v>2026-W42-Mon</x:v>
+      </x:c>
+      <x:c r="C3" s="2" t="str">
+        <x:v>5868491</x:v>
+      </x:c>
+      <x:c r="D3" s="2" t="str">
+        <x:v>jp-new-ryotaroito</x:v>
+      </x:c>
+      <x:c r="E3" s="2" t="str">
+        <x:v>伊藤涼太郎</x:v>
+      </x:c>
+      <x:c r="F3" s="2" t="str">
+        <x:v>Ryotaro Ito</x:v>
+      </x:c>
+      <x:c r="G3" s="2" t="str">
+        <x:v>Segunda Division</x:v>
+      </x:c>
+      <x:c r="H3" s="2" t="str">
+        <x:v>Real Valladolid</x:v>
+      </x:c>
+      <x:c r="I3" s="2" t="n">
+        <x:v>10281</x:v>
+      </x:c>
+      <x:c r="J3" s="2" t="str">
+        <x:v>Real Valladolid</x:v>
+      </x:c>
+      <x:c r="K3" s="2" t="n">
+        <x:v>10281</x:v>
+      </x:c>
+      <x:c r="L3" s="2" t="str">
+        <x:v>Albacete</x:v>
+      </x:c>
+      <x:c r="M3" s="2" t="n">
+        <x:v>8393</x:v>
+      </x:c>
+      <x:c r="N3" s="2" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O3" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P3" s="2" t="d">
+        <x:v>2026-10-12T12:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="Q3" s="2" t="d">
+        <x:v>2026-10-12T12:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="R3" s="2" t="str">
+        <x:v>Not in match squad</x:v>
+      </x:c>
+      <x:c r="S3" s="2"/>
+      <x:c r="T3" s="2"/>
+      <x:c r="U3" s="2"/>
+      <x:c r="V3" s="2"/>
+      <x:c r="W3" s="2"/>
+      <x:c r="X3" s="2"/>
+      <x:c r="Y3" s="2"/>
+      <x:c r="Z3" s="2" t="str"/>
+      <x:c r="AA3" s="2" t="str">
+        <x:v>https://www.fotmob.com/matches/albacete-vs-real-valladolid/2vti1w#5868491</x:v>
+      </x:c>
+      <x:c r="AB3" s="2" t="str">
+        <x:v>2026-10-13</x:v>
+      </x:c>
+      <x:c r="AC3" s="2" t="str">
+        <x:v>Verified match squad</x:v>
+      </x:c>
+      <x:c r="AD3" s="2" t="str">
+        <x:v>Squad independently checked: https://www.realvalladolid.es/partidos/temporada-2026-2027-laliga-hypermotion-9-real-valladolid-cf-vs-albacete-bp-3398; reason not inferred</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa8752709ca84aaa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13642,7 +13994,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5238542a150e4e94"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4507c3d96a344e12"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14344,7 +14696,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R53480e3e0d3049ff"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59d1f52892c248ef"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18616,7 +18968,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f73fe7e5cea4338"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb703f46094774d6b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23028,7 +23380,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra35cc87aff464c9f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40a9fd203e834bd6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23070,101 +23422,267 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
-      <x:c r="A1" s="4" t="str">
+      <x:c r="A1" s="6" t="str">
         <x:v>week</x:v>
       </x:c>
-      <x:c r="B1" s="4" t="str">
+      <x:c r="B1" s="6" t="str">
         <x:v>day_sheet</x:v>
       </x:c>
-      <x:c r="C1" s="4" t="str">
+      <x:c r="C1" s="6" t="str">
         <x:v>match_id</x:v>
       </x:c>
-      <x:c r="D1" s="4" t="str">
+      <x:c r="D1" s="6" t="str">
         <x:v>player_id</x:v>
       </x:c>
-      <x:c r="E1" s="4" t="str">
+      <x:c r="E1" s="6" t="str">
         <x:v>name_ja</x:v>
       </x:c>
-      <x:c r="F1" s="4" t="str">
+      <x:c r="F1" s="6" t="str">
         <x:v>name_en</x:v>
       </x:c>
-      <x:c r="G1" s="4" t="str">
+      <x:c r="G1" s="6" t="str">
         <x:v>league</x:v>
       </x:c>
-      <x:c r="H1" s="4" t="str">
+      <x:c r="H1" s="6" t="str">
         <x:v>club</x:v>
       </x:c>
-      <x:c r="I1" s="4" t="str">
+      <x:c r="I1" s="6" t="str">
         <x:v>club_id</x:v>
       </x:c>
-      <x:c r="J1" s="4" t="str">
+      <x:c r="J1" s="6" t="str">
         <x:v>home</x:v>
       </x:c>
-      <x:c r="K1" s="4" t="str">
+      <x:c r="K1" s="6" t="str">
         <x:v>home_id</x:v>
       </x:c>
-      <x:c r="L1" s="4" t="str">
+      <x:c r="L1" s="6" t="str">
         <x:v>away</x:v>
       </x:c>
-      <x:c r="M1" s="4" t="str">
+      <x:c r="M1" s="6" t="str">
         <x:v>away_id</x:v>
       </x:c>
-      <x:c r="N1" s="4" t="str">
+      <x:c r="N1" s="6" t="str">
         <x:v>home_goals</x:v>
       </x:c>
-      <x:c r="O1" s="4" t="str">
+      <x:c r="O1" s="6" t="str">
         <x:v>away_goals</x:v>
       </x:c>
-      <x:c r="P1" s="4" t="str">
+      <x:c r="P1" s="6" t="str">
         <x:v>kickoff_local</x:v>
       </x:c>
-      <x:c r="Q1" s="4" t="str">
+      <x:c r="Q1" s="6" t="str">
         <x:v>kickoff_jst</x:v>
       </x:c>
-      <x:c r="R1" s="4" t="str">
+      <x:c r="R1" s="6" t="str">
         <x:v>status</x:v>
       </x:c>
-      <x:c r="S1" s="4" t="str">
+      <x:c r="S1" s="6" t="str">
         <x:v>minutes</x:v>
       </x:c>
-      <x:c r="T1" s="4" t="str">
+      <x:c r="T1" s="6" t="str">
         <x:v>goals</x:v>
       </x:c>
-      <x:c r="U1" s="4" t="str">
+      <x:c r="U1" s="6" t="str">
         <x:v>assists</x:v>
       </x:c>
-      <x:c r="V1" s="4" t="str">
+      <x:c r="V1" s="6" t="str">
         <x:v>own_goals</x:v>
       </x:c>
-      <x:c r="W1" s="4" t="str">
+      <x:c r="W1" s="6" t="str">
         <x:v>yellow_cards</x:v>
       </x:c>
-      <x:c r="X1" s="4" t="str">
+      <x:c r="X1" s="6" t="str">
         <x:v>red_cards</x:v>
       </x:c>
-      <x:c r="Y1" s="4" t="str">
+      <x:c r="Y1" s="6" t="str">
         <x:v>rating</x:v>
       </x:c>
-      <x:c r="Z1" s="4" t="str">
+      <x:c r="Z1" s="6" t="str">
         <x:v>rating_provider</x:v>
       </x:c>
-      <x:c r="AA1" s="4" t="str">
+      <x:c r="AA1" s="6" t="str">
         <x:v>source_url</x:v>
       </x:c>
-      <x:c r="AB1" s="4" t="str">
+      <x:c r="AB1" s="6" t="str">
         <x:v>verified_at</x:v>
       </x:c>
-      <x:c r="AC1" s="4" t="str">
+      <x:c r="AC1" s="6" t="str">
         <x:v>verification_status</x:v>
       </x:c>
-      <x:c r="AD1" s="4" t="str">
+      <x:c r="AD1" s="6" t="str">
         <x:v>notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="25" customHeight="1">
+      <x:c r="A2" s="2" t="str">
+        <x:v>2026-W42</x:v>
+      </x:c>
+      <x:c r="B2" s="2" t="str">
+        <x:v>2026-W42-Mon</x:v>
+      </x:c>
+      <x:c r="C2" s="2" t="str">
+        <x:v>5795468</x:v>
+      </x:c>
+      <x:c r="D2" s="2" t="str">
+        <x:v>jp-007</x:v>
+      </x:c>
+      <x:c r="E2" s="2" t="str">
+        <x:v>坂元達裕</x:v>
+      </x:c>
+      <x:c r="F2" s="2" t="str">
+        <x:v>Tatsuhiro Sakamoto</x:v>
+      </x:c>
+      <x:c r="G2" s="2" t="str">
+        <x:v>Premier League</x:v>
+      </x:c>
+      <x:c r="H2" s="2" t="str">
+        <x:v>Coventry City</x:v>
+      </x:c>
+      <x:c r="I2" s="2" t="n">
+        <x:v>8669</x:v>
+      </x:c>
+      <x:c r="J2" s="2" t="str">
+        <x:v>Coventry City</x:v>
+      </x:c>
+      <x:c r="K2" s="2" t="n">
+        <x:v>8669</x:v>
+      </x:c>
+      <x:c r="L2" s="2" t="str">
+        <x:v>Newcastle United</x:v>
+      </x:c>
+      <x:c r="M2" s="2" t="n">
+        <x:v>10261</x:v>
+      </x:c>
+      <x:c r="N2" s="2" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="O2" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P2" s="2" t="d">
+        <x:v>2026-10-12T19:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="Q2" s="2" t="d">
+        <x:v>2026-10-12T19:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="R2" s="2" t="str">
+        <x:v>Substitute</x:v>
+      </x:c>
+      <x:c r="S2" s="2" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="T2" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U2" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="V2" s="2"/>
+      <x:c r="W2" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X2" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Y2" s="2" t="n">
+        <x:v>6.5</x:v>
+      </x:c>
+      <x:c r="Z2" s="2" t="str">
+        <x:v>FotMob</x:v>
+      </x:c>
+      <x:c r="AA2" s="2" t="str">
+        <x:v>https://www.fotmob.com/matches/coventry-city-vs-newcastle-united/2yooc8#5795468</x:v>
+      </x:c>
+      <x:c r="AB2" s="2" t="str">
+        <x:v>2026-10-13</x:v>
+      </x:c>
+      <x:c r="AC2" s="2" t="str">
+        <x:v>Verified match record</x:v>
+      </x:c>
+      <x:c r="AD2" s="2" t="str">
+        <x:v>Cross-checked score and goal events: https://www.newcastleunited.com/en/news/coventry-city-a-26-27-report; minutes, assists, cards and rating: FotMob</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="25" customHeight="1">
+      <x:c r="A3" s="2" t="str">
+        <x:v>2026-W42</x:v>
+      </x:c>
+      <x:c r="B3" s="2" t="str">
+        <x:v>2026-W42-Mon</x:v>
+      </x:c>
+      <x:c r="C3" s="2" t="str">
+        <x:v>5868491</x:v>
+      </x:c>
+      <x:c r="D3" s="2" t="str">
+        <x:v>jp-new-ryotaroito</x:v>
+      </x:c>
+      <x:c r="E3" s="2" t="str">
+        <x:v>伊藤涼太郎</x:v>
+      </x:c>
+      <x:c r="F3" s="2" t="str">
+        <x:v>Ryotaro Ito</x:v>
+      </x:c>
+      <x:c r="G3" s="2" t="str">
+        <x:v>Segunda Division</x:v>
+      </x:c>
+      <x:c r="H3" s="2" t="str">
+        <x:v>Real Valladolid</x:v>
+      </x:c>
+      <x:c r="I3" s="2" t="n">
+        <x:v>10281</x:v>
+      </x:c>
+      <x:c r="J3" s="2" t="str">
+        <x:v>Real Valladolid</x:v>
+      </x:c>
+      <x:c r="K3" s="2" t="n">
+        <x:v>10281</x:v>
+      </x:c>
+      <x:c r="L3" s="2" t="str">
+        <x:v>Albacete</x:v>
+      </x:c>
+      <x:c r="M3" s="2" t="n">
+        <x:v>8393</x:v>
+      </x:c>
+      <x:c r="N3" s="2" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O3" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P3" s="2" t="d">
+        <x:v>2026-10-12T12:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="Q3" s="2" t="d">
+        <x:v>2026-10-12T12:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="R3" s="2" t="str">
+        <x:v>Not in match squad</x:v>
+      </x:c>
+      <x:c r="S3" s="2"/>
+      <x:c r="T3" s="2"/>
+      <x:c r="U3" s="2"/>
+      <x:c r="V3" s="2"/>
+      <x:c r="W3" s="2"/>
+      <x:c r="X3" s="2"/>
+      <x:c r="Y3" s="2"/>
+      <x:c r="Z3" s="2" t="str"/>
+      <x:c r="AA3" s="2" t="str">
+        <x:v>https://www.fotmob.com/matches/albacete-vs-real-valladolid/2vti1w#5868491</x:v>
+      </x:c>
+      <x:c r="AB3" s="2" t="str">
+        <x:v>2026-10-13</x:v>
+      </x:c>
+      <x:c r="AC3" s="2" t="str">
+        <x:v>Verified match squad</x:v>
+      </x:c>
+      <x:c r="AD3" s="2" t="str">
+        <x:v>Squad independently checked: https://www.realvalladolid.es/partidos/temporada-2026-2027-laliga-hypermotion-9-real-valladolid-cf-vs-albacete-bp-3398; reason not inferred</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R39a18886d86a48c6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf6018d86fa694a30"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23280,7 +23798,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R373a429f6e8d42f9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5111e491687040b5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23809,7 +24327,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4a0d024bc6242c5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbeadc3f9dd504ea2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23913,7 +24431,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1fe2200253334ab7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa8a3aa2cf9d4b70"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>